<commit_message>
docs: capture ritual — handoff refresh + session dossier + Amber gauge rule
- GOOD-MORNING: two names, §B (this session), §C queue (go straight to build-out;
  RAG error/warning/info still Legacy-drifted before Alert/Banner/Toast).
- _LIVE-STATE: new latest-delta + refreshed marker (build rebind, leak gate R-D17,
  RAG green R-D18, ADR-0010, Icon button).
- _DECISION-HISTORY/2026-07-20-button-rebind-legacy-leak-gate.md — narrative dossier.
- _RUNBOOK-context-gauge: proactively surface the gauge at AMBER, don't wait to be
  asked (Dave — "I would set it at amber too"). Mirrored to memory feedback-context-gauge.
- Itinerary: Icon button Gap -> Gated (39 gated / 39 P1 gaps).

Build green 36/36; STAND-002 reachable; GOOD-MORNING structure intact.
</commit_message>
<xml_diff>
--- a/reviews/ITINERARY-2026-07-14-apollo-component-library.xlsx
+++ b/reviews/ITINERARY-2026-07-14-apollo-component-library.xlsx
@@ -825,17 +825,17 @@
       </c>
       <c r="E6" s="8" t="inlineStr">
         <is>
-          <t>Gap</t>
+          <t>Gated</t>
         </is>
       </c>
       <c r="F6" s="9" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P0</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>1 Foundations</t>
+          <t>0 Have</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr">
@@ -845,7 +845,7 @@
       </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t>Reliability-critical; used everywhere.</t>
+          <t>Reviewed + gated 2026-07-20 — Mono button/* ladder, real sprite glyphs, icon-015 4.5:1</t>
         </is>
       </c>
     </row>

</xml_diff>